<commit_message>
sửa dữ liệu excel
</commit_message>
<xml_diff>
--- a/file du lieu.xlsx
+++ b/file du lieu.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\quản lý công việc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\quan ly cong viec\quan_ly_cong_viec\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFCCE125-701B-4732-8E95-69CC73EF103B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B68238-C6BC-42BD-8E5E-D989C6536DCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{E043318D-88E5-4774-B12C-14EEF7D47615}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="23040" windowHeight="12120" xr2:uid="{E043318D-88E5-4774-B12C-14EEF7D47615}"/>
   </bookViews>
   <sheets>
     <sheet name="Tổng hợp" sheetId="1" r:id="rId1"/>
@@ -479,6 +479,15 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -486,15 +495,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2404,84 +2404,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:45" s="1" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20" t="s">
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20" t="s">
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20" t="s">
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20" t="s">
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
-      <c r="S1" s="20" t="s">
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
+      <c r="S1" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="20"/>
-      <c r="U1" s="20"/>
-      <c r="V1" s="20" t="s">
+      <c r="T1" s="17"/>
+      <c r="U1" s="17"/>
+      <c r="V1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="W1" s="20"/>
-      <c r="X1" s="20"/>
-      <c r="Y1" s="20" t="s">
+      <c r="W1" s="17"/>
+      <c r="X1" s="17"/>
+      <c r="Y1" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="Z1" s="20"/>
-      <c r="AA1" s="20"/>
-      <c r="AB1" s="17" t="s">
+      <c r="Z1" s="17"/>
+      <c r="AA1" s="17"/>
+      <c r="AB1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="AC1" s="18"/>
-      <c r="AD1" s="19"/>
-      <c r="AE1" s="17" t="s">
+      <c r="AC1" s="21"/>
+      <c r="AD1" s="22"/>
+      <c r="AE1" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="AF1" s="18"/>
-      <c r="AG1" s="19"/>
-      <c r="AH1" s="17" t="s">
+      <c r="AF1" s="21"/>
+      <c r="AG1" s="22"/>
+      <c r="AH1" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="AI1" s="18"/>
-      <c r="AJ1" s="19"/>
-      <c r="AK1" s="17" t="s">
+      <c r="AI1" s="21"/>
+      <c r="AJ1" s="22"/>
+      <c r="AK1" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="AL1" s="18"/>
-      <c r="AM1" s="19"/>
-      <c r="AN1" s="17" t="s">
+      <c r="AL1" s="21"/>
+      <c r="AM1" s="22"/>
+      <c r="AN1" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="AO1" s="18"/>
-      <c r="AP1" s="19"/>
-      <c r="AQ1" s="17" t="s">
+      <c r="AO1" s="21"/>
+      <c r="AP1" s="22"/>
+      <c r="AQ1" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="AR1" s="18"/>
-      <c r="AS1" s="19"/>
+      <c r="AR1" s="21"/>
+      <c r="AS1" s="22"/>
     </row>
     <row r="2" spans="1:45" s="1" customFormat="1" ht="67.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="22"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2" t="s">
         <v>15</v>
       </c>
@@ -2670,7 +2670,7 @@
         <v>46301</v>
       </c>
       <c r="V3" s="5">
-        <v>15</v>
+        <v>155</v>
       </c>
       <c r="W3" s="5">
         <v>12</v>
@@ -4617,12 +4617,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="P1:R1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="J1:L1"/>
-    <mergeCell ref="M1:O1"/>
     <mergeCell ref="AK1:AM1"/>
     <mergeCell ref="AN1:AP1"/>
     <mergeCell ref="AQ1:AS1"/>
@@ -4632,6 +4626,12 @@
     <mergeCell ref="AB1:AD1"/>
     <mergeCell ref="AE1:AG1"/>
     <mergeCell ref="AH1:AJ1"/>
+    <mergeCell ref="P1:R1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="J1:L1"/>
+    <mergeCell ref="M1:O1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="46" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>